<commit_message>
docs: relatorio operacional revisado (secao 8 de validacao; notas nas secoes 4.2, 6.2, 6.3, 6.5); planilha com os 4 FP sem explicacao
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frente_ocsvm/revisao/paradas_para_revisao.xlsx
+++ b/frente_ocsvm/revisao/paradas_para_revisao.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paradas para revisão" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trips curados (referência)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alertas sem explicação" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -479,7 +480,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Classificação: escolher na lista (Programada / Operacional (não programada, sem falha) / Falha de equipamento / Não sei).</t>
+          <t>Classificação: escolher na lista (Programada / Operacional não programada (sem falha) / Falha de equipamento / Não sei).</t>
         </is>
       </c>
     </row>
@@ -515,14 +516,31 @@
       <c r="A10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>Exemplo de preenchimento (fictício):</t>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Segundo pedido: a aba 'Alertas sem explicação' tem 4 alertas do modelo em que nenhum sensor mostrou variação. A máquina seguiu operando. O que aconteceu nesses intervalos?</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Classificação: escolher na lista (Manobra ou intervenção operacional / Problema de instrumento/sensor / Evento de processo (sem falha) / Nada de anormal / Não sei).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Exemplo de preenchimento (fictício):</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Classificação = Programada · Motivo = Parada para lavagem do compressor · Fonte = Livro de turno de 12/03/2025</t>
         </is>
@@ -1378,7 +1396,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="G2:G32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Programada,Operacional (não programada, sem falha),Falha de equipamento,Não sei"</formula1>
+      <formula1>"Programada,Operacional não programada (sem falha),Falha de equipamento,Não sei"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1659,4 +1677,189 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Nº</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Início (Brasília)</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Fim (Brasília)</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Duração (h)</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Sinais que acenderam no modelo</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Alarmes do catálogo de 2 h antes ao fim</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Classificação</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Motivo / observação</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Fonte</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>45671.62291666667</v>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>45671.66770833333</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>temperatura de mancal, vibração de mancal, alarme recente do catálogo (24 h)</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>PAL_6240315 (TC_33003A - Pressão Baixa Gás Comb., LOW)</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr"/>
+      <c r="H2" s="6" t="inlineStr"/>
+      <c r="I2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>45681.40416666667</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>45681.44201388889</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>temperatura de mancal, vibração de mancal, alarme recente do catálogo (24 h)</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>PAL_6240315 (TC_33003A - Pressão Baixa Gás Comb., LOW); PDAL_6240302 (TC_33003A - PrDif.Bx.Gás Linha Balanc., LOW)</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr"/>
+      <c r="H3" s="6" t="inlineStr"/>
+      <c r="I3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>45709.01909722222</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>45709.06909722222</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>vibração de mancal, pressão de óleo, alarme recente do catálogo (24 h)</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>PAL_6240315 (TC_33003A - Pressão Baixa Gás Comb., LOW); PI_6240319_AL (TC_33003A - Falha PI Gás Motor p/Partida, LOW)</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>46090.38020833334</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>46090.41701388889</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>vibração de mancal, alarme recente do catálogo (24 h)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>PAL_6240315 (TC_33003A - Pressão Baixa Gás Comb., LOW)</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="G2:G5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Manobra ou intervenção operacional,Problema de instrumento/sensor,Evento de processo (sem falha),Nada de anormal,Não sei"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>